<commit_message>
docs(coach): lexique Sheet à jour + onglet Notes.
Familles 01–13 soft, marges D alignées code, notes coach (éducatifs, calendrier S-6/S-7, pièges).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/coach-ligne/lexique-sheet-myswym.xlsx
+++ b/docs/coach-ligne/lexique-sheet-myswym.xlsx
@@ -13,6 +13,7 @@
     <sheet name="4 · Rédiger une séance" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5 · Familles onglets" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6 · Calcul D (indicatif)" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7 · Notes" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1607,11 +1608,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1744,17 +1745,119 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>07–13 …</t>
+          <t>07 Oly-Half-Full crawl</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Oly / OW — pas encore soft</t>
+          <t>Inter crawl · Oly/Half/Full</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Composeur pour l’instant</t>
+          <t>Oui si Premium + T100</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>08 Oly-Half-Full 4 nages</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Inter 4n / Avancé · Oly/Half/Full</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Oui si Premium + T100</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>09 OW courte deb crawl</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Débutant · OW courte</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Non (débutant)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>10 OW courte crawl</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Inter crawl · OW courte</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Oui si Premium + T100</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>11 OW courte 4 nages</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Inter 4n / Avancé · OW courte</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Oui si Premium + T100</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>12 OW moy-long crawl</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Inter crawl · OW moy/long</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Oui si Premium + T100</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>13 OW moy-long 4 nages</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Inter 4n / Avancé · OW moy/long</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Oui si Premium + T100</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1879,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="28" customWidth="1" min="3" max="3"/>
     <col width="36" customWidth="1" min="4" max="4"/>
   </cols>
@@ -1784,7 +1887,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Comment l’app calcule D (tu peux faire corriger les marges)</t>
+          <t>Comment l’app calcule D (marges = code pace-placeholders.js)</t>
         </is>
       </c>
     </row>
@@ -1818,7 +1921,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>~1,35 × T100 (Z1)</t>
+          <t>zone easy (Z1)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -1840,7 +1943,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>milieu Z1/Z2–Z3</t>
+          <t>milieu easy / seuil</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -1862,7 +1965,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>~1,08–1,12 × T100</t>
+          <t>zone threshold</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1884,7 +1987,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>proche / sous T100</t>
+          <t>proche / un cran sous sprint</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1906,7 +2009,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>plus vite que VO2</t>
+          <t>plus vite que VO2 (max court)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1923,7 +2026,7 @@
     <row r="9" ht="50" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Formule : D = arrondi 5 s ( T100 × mult × (distance_rep/100) + marge ). Distance lue sur la ligne (8 × 50 m → 50). Débutant / sans T100 / non Premium → {D:} devient « repos 30 s ».</t>
+          <t>Formule : D = arrondi 5 s ( T100 × mult × (distance_rep/100) + marge ). Distance lue sur la ligne (8 × 50 m → 50). Débutant / sans T100 / non Premium → {D:} devient « repos 30 s » ; {@:} retiré.</t>
         </is>
       </c>
     </row>
@@ -1934,4 +2037,288 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="78" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Notes coach — pièges, colonnes Sheet, calendrier vers J</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sujet</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Règle</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Détail</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="48" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Colonne Notes (onglet Éducatifs)</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Libre — pour toi, pas un filtre app</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>L’app lit Nom, Nage, niveaux oui/non, utilité, comment, Matériel optionnel, Garder. La colonne Notes du Sheet éducatifs n’oriente pas le tirage : c’est ton mémo coach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="48" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Garder = oui</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Seul filtre « actif »</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Un éducatif avec Garder ≠ oui n’entre jamais dans le tirage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Matériel optionnel</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>et/ou = alternatives</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Ne gate pas le choix de l’éducatif. Remplit {matériel} seulement si ∩ inventaire nageur. Jamais pull-buoy + palmes sur la même ligne d’exercice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="48" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Débutant</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Jamais {D:} / {@:}</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Sur 01 / 04 / 09 : mots souple / moyen + repos … s. Sinon l’app force repos 30 s.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="48" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Inter / Avancé + pace</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Premium + T100</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Sans T100 ou hors Premium → même fallback (repos / token retiré).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="48" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>D fixe vs {D:}</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Ne pas mélanger</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Une ligne avec D2' (horloge bassin) + {D:seuil} = conflit. Un seul type de départ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>4 nages + éducatifs</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>1 éducatif / nage</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Écrire « 4 nages » + « éducatif(s) » → pap → dos → brasse → crawl. Distances Sheet inchangées.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Anti-doublon éducatif</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Pas 2× d’affilée</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Dernier éducatif exclu en dur ; variété sur ~5 derniers si le pool le permet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Calendrier vers J (tri / OW)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>S-6 allégée · S-7 test</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Depuis J : S0 course (max 2 séances) · S-1 allégée · S-2→S-5 travail · S-6 allégée cycle · S-7 test · puis 6 travail entre chaque couple. Pas de test/allégée cycle avant S-6. Début de plan : 2 sem. travail avant le 1er couple.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="48" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Planning app</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Pastille = progression</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>« Cette semaine » avance avec les semaines validées (Semaine 2 → S-n−1), pas seulement le calendrier civil.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Soft-branch 01–13</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pas de fallback composeur</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Familles soft = Sheet obligatoire. Diplômes restent composeur (pas d’onglet Sheet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="48" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Réf. séance</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>UI n° ≠ ligne Sheet</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Pastille Réf. 01-42 = onglet + ligne n. « Séance n°6 » = compteur nageur (validations).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="48" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Orthographe tokens</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Exact</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>{D:endurance} {D:VO2} — pas d’espace ; alias (moyen, vite…) OK mais préfère le canonique.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="48" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Regen Excel</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>python3 docs/coach-ligne/build_lexique_sheet.py</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Régénère lexique-sheet-myswym.xlsx. Coller / partager hors repo si tu travailles surtout sur Google Sheet.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>